<commit_message>
Planilha de Campanhas: regra da janela e rotulagem no Como usar
A regra (entra tudo que gastou na janela, pausado inclusive; achado com
fonte + janela + status) existia so nas skills — quem usa a planilha sem IA
nao ficava sabendo. Agora esta no passo a passo do gabarito.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/planilhas/Auditoria de Campanhas - V4.xlsx
+++ b/planilhas/Auditoria de Campanhas - V4.xlsx
@@ -586,7 +586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -652,82 +652,96 @@
     <row r="11">
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>2. Comece pela aba Fundamentos (vale para todos os canais).</t>
+          <t>2. Defina a janela auditada (ex.: últimos 30 ou 60 dias) e use a mesma em todas as fontes. Entra na análise tudo que GASTOU dentro da janela — inclusive campanha ou anúncio já pausado (verba queimada antes da pausa é achado). O que não gastou nada na janela fica fora.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>3. Depois audite cada canal ativo na aba correspondente. Pule canais que o cliente não usa (marque N/A).</t>
+          <t>3. Anote em cada observação a fonte, a janela e o status do que foi visto (ex.: Google Ads · termos de pesquisa · 60d · R$ 500 · pausados) — é o que permite conferir o ponto depois.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>4. Para cada item: leia 'Como auditar', compare com o 'Benchmark', defina o Status e anote em Observações.</t>
+          <t>4. Comece pela aba Fundamentos (vale para todos os canais).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>5. Quando o Status for Ajustar/Crítico, registre o plano na coluna 'Como corrigir' como guia.</t>
+          <t>5. Depois audite cada canal ativo na aba correspondente. Pule canais que o cliente não usa (marque N/A).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>6. Acompanhe o progresso na aba Resumo (preenche automaticamente).</t>
+          <t>6. Para cada item: leia 'Como auditar', compare com o 'Benchmark', defina o Status e anote em Observações.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>7. Quando o Status for Ajustar/Crítico, registre o plano na coluna 'Como corrigir' como guia.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>8. Acompanhe o progresso na aba Resumo (preenche automaticamente).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="3" t="inlineStr">
         <is>
           <t>Como ler as colunas</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="4" t="inlineStr">
-        <is>
-          <t>•  Como auditar — onde olhar e o que verificar em cada ponto.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="4" t="inlineStr">
-        <is>
-          <t>•  Benchmark / Referência 2026 — número de comparação. '(validar)' = confirmar no contexto do cliente.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>•  Como corrigir — o que fazer quando o ponto está fora do esperado.</t>
+          <t>•  Como auditar — onde olhar e o que verificar em cada ponto.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>•  Criticidade — Crítico (resolver já) · Importante (resolver no ciclo) · Bom ter (ganho marginal).</t>
+          <t>•  Benchmark / Referência 2026 — número de comparação. '(validar)' = confirmar no contexto do cliente.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>•  Status — Pendente / OK / Ajustar / Crítico / N/A (menu suspenso). A aba Resumo conta sozinha.</t>
+          <t>•  Como corrigir — o que fazer quando o ponto está fora do esperado.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>•  Criticidade — Crítico (resolver já) · Importante (resolver no ciclo) · Bom ter (ganho marginal).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>•  Status — Pendente / OK / Ajustar / Crítico / N/A (menu suspenso). A aba Resumo conta sozinha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t>•  Coluna ✓ — selecione o ✓ para marcar o item como revisado (fica verde).</t>
         </is>

</xml_diff>